<commit_message>
Update EquiArena template font styling validation
</commit_message>
<xml_diff>
--- a/app/templates/Template_EquiArena.xlsx
+++ b/app/templates/Template_EquiArena.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2FC55B9-D11A-488B-89BA-2A69A2386188}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50DF63C9-7A68-4BFC-B408-A34A077C948A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="723" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -734,7 +734,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="139">
+  <cellXfs count="137">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="2" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -766,479 +766,473 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="17" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="17" fontId="6" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="18" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="19" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="20" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="18" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="18" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="19" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="20" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="13" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="20" fontId="8" fillId="3" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="16" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="18" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="16" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="16" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" indent="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" indent="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" indent="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="17" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyProtection="1">
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="22" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="23" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="21" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="18" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="18" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="18" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="22" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="21" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="17" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="17" fontId="6" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="22" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="23" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="21" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="22" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="21" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="18" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="19" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="20" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="18" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="10" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="18" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="19" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="20" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="2" fontId="13" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="20" fontId="8" fillId="3" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="16" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="18" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="2" fontId="16" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="16" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" indent="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" indent="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" indent="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="17" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="18" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="18" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="18" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyProtection="1">
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0" hidden="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -2131,388 +2125,388 @@
   <dimension ref="A1:N56"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.33203125" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.88671875" style="19" customWidth="1"/>
-    <col min="2" max="2" width="9.109375" style="19" customWidth="1"/>
-    <col min="3" max="3" width="5.6640625" style="19" customWidth="1"/>
-    <col min="4" max="4" width="10.109375" style="19" customWidth="1"/>
-    <col min="5" max="5" width="8.109375" style="19" customWidth="1"/>
-    <col min="6" max="6" width="11.33203125" style="19" customWidth="1"/>
-    <col min="7" max="7" width="11.109375" style="19" customWidth="1"/>
-    <col min="8" max="10" width="13" style="19" customWidth="1"/>
-    <col min="11" max="11" width="6.44140625" style="19" customWidth="1"/>
-    <col min="12" max="12" width="9.44140625" style="19" customWidth="1"/>
-    <col min="13" max="14" width="10.6640625" style="19" customWidth="1"/>
-    <col min="15" max="16384" width="10.33203125" style="19"/>
+    <col min="1" max="1" width="6.88671875" style="18" customWidth="1"/>
+    <col min="2" max="2" width="9.109375" style="18" customWidth="1"/>
+    <col min="3" max="3" width="5.6640625" style="18" customWidth="1"/>
+    <col min="4" max="4" width="10.109375" style="18" customWidth="1"/>
+    <col min="5" max="5" width="8.109375" style="18" customWidth="1"/>
+    <col min="6" max="6" width="11.33203125" style="18" customWidth="1"/>
+    <col min="7" max="7" width="11.109375" style="18" customWidth="1"/>
+    <col min="8" max="10" width="13" style="18" customWidth="1"/>
+    <col min="11" max="11" width="6.44140625" style="18" customWidth="1"/>
+    <col min="12" max="12" width="9.44140625" style="18" customWidth="1"/>
+    <col min="13" max="14" width="10.6640625" style="18" customWidth="1"/>
+    <col min="15" max="16384" width="10.33203125" style="18"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="15"/>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="18"/>
+      <c r="A1" s="14"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="17"/>
     </row>
     <row r="2" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="20"/>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
-      <c r="I2" s="22"/>
-      <c r="J2" s="23"/>
+      <c r="A2" s="19"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
+      <c r="I2" s="21"/>
+      <c r="J2" s="22"/>
     </row>
     <row r="3" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="20"/>
-      <c r="B3" s="21"/>
-      <c r="C3" s="21"/>
-      <c r="D3" s="21"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="22"/>
-      <c r="I3" s="22"/>
-      <c r="J3" s="23"/>
+      <c r="A3" s="19"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
+      <c r="G3" s="21"/>
+      <c r="H3" s="21"/>
+      <c r="I3" s="21"/>
+      <c r="J3" s="22"/>
     </row>
     <row r="4" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="20"/>
-      <c r="B4" s="21"/>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
-      <c r="G4" s="22"/>
-      <c r="H4" s="22"/>
-      <c r="I4" s="22"/>
-      <c r="J4" s="23"/>
+      <c r="A4" s="19"/>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="21"/>
+      <c r="H4" s="21"/>
+      <c r="I4" s="21"/>
+      <c r="J4" s="22"/>
     </row>
     <row r="5" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="24"/>
-      <c r="B5" s="25"/>
-      <c r="C5" s="25"/>
-      <c r="D5" s="25"/>
-      <c r="E5" s="25"/>
-      <c r="F5" s="25"/>
-      <c r="G5" s="25"/>
-      <c r="H5" s="25"/>
-      <c r="I5" s="25"/>
-      <c r="J5" s="26"/>
+      <c r="A5" s="23"/>
+      <c r="B5" s="24"/>
+      <c r="C5" s="24"/>
+      <c r="D5" s="24"/>
+      <c r="E5" s="24"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="24"/>
+      <c r="H5" s="24"/>
+      <c r="I5" s="24"/>
+      <c r="J5" s="25"/>
     </row>
     <row r="6" spans="1:13" ht="5.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="27"/>
-      <c r="B6" s="27"/>
-      <c r="C6" s="27"/>
-      <c r="D6" s="27"/>
-      <c r="E6" s="27"/>
-      <c r="F6" s="27"/>
-      <c r="G6" s="27"/>
-      <c r="H6" s="27"/>
-      <c r="I6" s="27"/>
-      <c r="J6" s="27"/>
+      <c r="A6" s="26"/>
+      <c r="B6" s="26"/>
+      <c r="C6" s="26"/>
+      <c r="D6" s="26"/>
+      <c r="E6" s="26"/>
+      <c r="F6" s="26"/>
+      <c r="G6" s="26"/>
+      <c r="H6" s="26"/>
+      <c r="I6" s="26"/>
+      <c r="J6" s="26"/>
     </row>
     <row r="7" spans="1:13" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="28" t="s">
+      <c r="A7" s="117" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="28"/>
-      <c r="C7" s="28"/>
-      <c r="D7" s="28"/>
-      <c r="E7" s="28"/>
-      <c r="F7" s="28"/>
-      <c r="G7" s="28"/>
-      <c r="H7" s="28"/>
-      <c r="I7" s="28"/>
-      <c r="J7" s="28"/>
-      <c r="M7" s="29"/>
+      <c r="B7" s="117"/>
+      <c r="C7" s="117"/>
+      <c r="D7" s="117"/>
+      <c r="E7" s="117"/>
+      <c r="F7" s="117"/>
+      <c r="G7" s="117"/>
+      <c r="H7" s="117"/>
+      <c r="I7" s="117"/>
+      <c r="J7" s="117"/>
+      <c r="M7" s="28"/>
     </row>
     <row r="8" spans="1:13" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="30" t="s">
+      <c r="A8" s="118" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="30"/>
-      <c r="C8" s="30"/>
-      <c r="D8" s="30"/>
-      <c r="E8" s="30"/>
-      <c r="F8" s="30"/>
-      <c r="G8" s="30"/>
-      <c r="H8" s="30"/>
-      <c r="I8" s="30"/>
-      <c r="J8" s="30"/>
+      <c r="B8" s="118"/>
+      <c r="C8" s="118"/>
+      <c r="D8" s="118"/>
+      <c r="E8" s="118"/>
+      <c r="F8" s="118"/>
+      <c r="G8" s="118"/>
+      <c r="H8" s="118"/>
+      <c r="I8" s="118"/>
+      <c r="J8" s="118"/>
     </row>
     <row r="9" spans="1:13" ht="6.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="31"/>
-      <c r="B9" s="31"/>
-      <c r="C9" s="31"/>
-      <c r="D9" s="31"/>
-      <c r="E9" s="31"/>
-      <c r="F9" s="31"/>
-      <c r="G9" s="31"/>
-      <c r="H9" s="31"/>
-      <c r="I9" s="31"/>
-      <c r="J9" s="31"/>
+      <c r="A9" s="27"/>
+      <c r="B9" s="27"/>
+      <c r="C9" s="27"/>
+      <c r="D9" s="27"/>
+      <c r="E9" s="27"/>
+      <c r="F9" s="27"/>
+      <c r="G9" s="27"/>
+      <c r="H9" s="27"/>
+      <c r="I9" s="27"/>
+      <c r="J9" s="27"/>
     </row>
     <row r="10" spans="1:13" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="32" t="s">
+      <c r="B10" s="131" t="s">
         <v>73</v>
       </c>
-      <c r="C10" s="32"/>
-      <c r="D10" s="32" t="s">
+      <c r="C10" s="131"/>
+      <c r="D10" s="131" t="s">
         <v>74</v>
       </c>
-      <c r="E10" s="32"/>
-      <c r="F10" s="32" t="s">
+      <c r="E10" s="131"/>
+      <c r="F10" s="131" t="s">
         <v>75</v>
       </c>
-      <c r="G10" s="32"/>
-      <c r="H10" s="32" t="s">
+      <c r="G10" s="131"/>
+      <c r="H10" s="131" t="s">
         <v>76</v>
       </c>
-      <c r="I10" s="32"/>
-      <c r="J10" s="33"/>
-      <c r="K10" s="34"/>
-      <c r="L10" s="34"/>
+      <c r="I10" s="131"/>
+      <c r="J10" s="29"/>
+      <c r="K10" s="30"/>
+      <c r="L10" s="30"/>
     </row>
     <row r="11" spans="1:13" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="35"/>
-      <c r="B11" s="32"/>
-      <c r="C11" s="32"/>
-      <c r="D11" s="32"/>
-      <c r="E11" s="32"/>
-      <c r="F11" s="32"/>
-      <c r="G11" s="32"/>
-      <c r="H11" s="32"/>
-      <c r="I11" s="32"/>
-      <c r="J11" s="36"/>
-      <c r="K11" s="34"/>
-      <c r="L11" s="34"/>
+      <c r="A11" s="31"/>
+      <c r="B11" s="131"/>
+      <c r="C11" s="131"/>
+      <c r="D11" s="131"/>
+      <c r="E11" s="131"/>
+      <c r="F11" s="131"/>
+      <c r="G11" s="131"/>
+      <c r="H11" s="131"/>
+      <c r="I11" s="131"/>
+      <c r="J11" s="32"/>
+      <c r="K11" s="30"/>
+      <c r="L11" s="30"/>
     </row>
     <row r="12" spans="1:13" ht="7.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="35"/>
-      <c r="B12" s="35"/>
-      <c r="C12" s="37"/>
-      <c r="D12" s="38"/>
-      <c r="E12" s="38"/>
-      <c r="F12" s="38"/>
-      <c r="G12" s="38"/>
-      <c r="H12" s="38"/>
-      <c r="I12" s="38"/>
-      <c r="J12" s="39"/>
-      <c r="K12" s="34"/>
-      <c r="L12" s="34"/>
+      <c r="A12" s="31"/>
+      <c r="B12" s="31"/>
+      <c r="C12" s="33"/>
+      <c r="D12" s="34"/>
+      <c r="E12" s="34"/>
+      <c r="F12" s="34"/>
+      <c r="G12" s="34"/>
+      <c r="H12" s="34"/>
+      <c r="I12" s="34"/>
+      <c r="J12" s="35"/>
+      <c r="K12" s="30"/>
+      <c r="L12" s="30"/>
     </row>
     <row r="13" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="40" t="s">
+      <c r="A13" s="122" t="s">
         <v>58</v>
       </c>
-      <c r="B13" s="41"/>
-      <c r="C13" s="41"/>
-      <c r="D13" s="41"/>
-      <c r="E13" s="41"/>
-      <c r="F13" s="41"/>
-      <c r="G13" s="41"/>
-      <c r="H13" s="41"/>
-      <c r="I13" s="41"/>
-      <c r="J13" s="42"/>
-      <c r="K13" s="34"/>
-      <c r="L13" s="34"/>
+      <c r="B13" s="123"/>
+      <c r="C13" s="123"/>
+      <c r="D13" s="123"/>
+      <c r="E13" s="123"/>
+      <c r="F13" s="123"/>
+      <c r="G13" s="123"/>
+      <c r="H13" s="123"/>
+      <c r="I13" s="123"/>
+      <c r="J13" s="124"/>
+      <c r="K13" s="30"/>
+      <c r="L13" s="30"/>
     </row>
     <row r="14" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="43" t="s">
+      <c r="A14" s="99" t="s">
         <v>61</v>
       </c>
-      <c r="B14" s="44"/>
-      <c r="C14" s="44"/>
-      <c r="D14" s="44"/>
-      <c r="E14" s="44"/>
-      <c r="F14" s="44"/>
-      <c r="G14" s="44"/>
-      <c r="H14" s="44"/>
-      <c r="I14" s="44"/>
-      <c r="J14" s="45"/>
-      <c r="K14" s="34"/>
-      <c r="L14" s="34"/>
+      <c r="B14" s="100"/>
+      <c r="C14" s="100"/>
+      <c r="D14" s="100"/>
+      <c r="E14" s="100"/>
+      <c r="F14" s="100"/>
+      <c r="G14" s="100"/>
+      <c r="H14" s="100"/>
+      <c r="I14" s="100"/>
+      <c r="J14" s="101"/>
+      <c r="K14" s="30"/>
+      <c r="L14" s="30"/>
     </row>
     <row r="15" spans="1:13" ht="6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="46"/>
-      <c r="B15" s="47"/>
-      <c r="C15" s="48"/>
-      <c r="D15" s="49"/>
-      <c r="E15" s="49"/>
-      <c r="F15" s="49"/>
-      <c r="G15" s="49"/>
-      <c r="H15" s="49"/>
-      <c r="I15" s="49"/>
-      <c r="J15" s="50"/>
-      <c r="K15" s="34"/>
-      <c r="L15" s="34"/>
+      <c r="A15" s="36"/>
+      <c r="B15" s="37"/>
+      <c r="C15" s="38"/>
+      <c r="D15" s="39"/>
+      <c r="E15" s="39"/>
+      <c r="F15" s="39"/>
+      <c r="G15" s="39"/>
+      <c r="H15" s="39"/>
+      <c r="I15" s="39"/>
+      <c r="J15" s="40"/>
+      <c r="K15" s="30"/>
+      <c r="L15" s="30"/>
     </row>
     <row r="16" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="51"/>
-      <c r="B16" s="52" t="s">
+      <c r="A16" s="41"/>
+      <c r="B16" s="125" t="s">
         <v>37</v>
       </c>
-      <c r="C16" s="52"/>
-      <c r="D16" s="52"/>
-      <c r="E16" s="53"/>
-      <c r="F16" s="54" t="s">
+      <c r="C16" s="125"/>
+      <c r="D16" s="125"/>
+      <c r="E16" s="42"/>
+      <c r="F16" s="126" t="s">
         <v>38</v>
       </c>
-      <c r="G16" s="54"/>
-      <c r="H16" s="53"/>
-      <c r="I16" s="55" t="s">
+      <c r="G16" s="126"/>
+      <c r="H16" s="42"/>
+      <c r="I16" s="102" t="s">
         <v>60</v>
       </c>
-      <c r="J16" s="56"/>
-      <c r="K16" s="34"/>
-      <c r="L16" s="34"/>
+      <c r="J16" s="105"/>
+      <c r="K16" s="30"/>
+      <c r="L16" s="30"/>
     </row>
     <row r="17" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="51"/>
-      <c r="B17" s="57" t="s">
+      <c r="A17" s="41"/>
+      <c r="B17" s="132" t="s">
         <v>80</v>
       </c>
-      <c r="C17" s="58"/>
-      <c r="D17" s="59"/>
-      <c r="E17" s="60"/>
-      <c r="F17" s="57" t="s">
+      <c r="C17" s="133"/>
+      <c r="D17" s="134"/>
+      <c r="E17" s="43"/>
+      <c r="F17" s="132" t="s">
         <v>81</v>
       </c>
-      <c r="G17" s="59"/>
-      <c r="H17" s="53"/>
-      <c r="I17" s="61"/>
-      <c r="J17" s="62"/>
-      <c r="K17" s="34"/>
-      <c r="L17" s="34"/>
+      <c r="G17" s="134"/>
+      <c r="H17" s="42"/>
+      <c r="I17" s="103"/>
+      <c r="J17" s="106"/>
+      <c r="K17" s="30"/>
+      <c r="L17" s="30"/>
     </row>
     <row r="18" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E18" s="60"/>
-      <c r="F18" s="60"/>
-      <c r="G18" s="60"/>
-      <c r="H18" s="53"/>
-      <c r="I18" s="63"/>
-      <c r="J18" s="64"/>
-      <c r="L18" s="34"/>
-      <c r="M18" s="65"/>
+      <c r="E18" s="43"/>
+      <c r="F18" s="43"/>
+      <c r="G18" s="43"/>
+      <c r="H18" s="42"/>
+      <c r="I18" s="104"/>
+      <c r="J18" s="107"/>
+      <c r="L18" s="30"/>
+      <c r="M18" s="44"/>
     </row>
     <row r="19" spans="1:14" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="66"/>
-      <c r="B19" s="60"/>
-      <c r="C19" s="60"/>
-      <c r="D19" s="53"/>
-      <c r="E19" s="60"/>
-      <c r="F19" s="36"/>
-      <c r="G19" s="60"/>
-      <c r="H19" s="53"/>
-      <c r="I19" s="60"/>
-      <c r="J19" s="67"/>
-      <c r="L19" s="34"/>
-      <c r="M19" s="65"/>
-    </row>
-    <row r="20" spans="1:14" s="71" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="68"/>
-      <c r="B20" s="69" t="s">
+      <c r="A19" s="45"/>
+      <c r="B19" s="43"/>
+      <c r="C19" s="43"/>
+      <c r="D19" s="42"/>
+      <c r="E19" s="43"/>
+      <c r="F19" s="32"/>
+      <c r="G19" s="43"/>
+      <c r="H19" s="42"/>
+      <c r="I19" s="43"/>
+      <c r="J19" s="46"/>
+      <c r="L19" s="30"/>
+      <c r="M19" s="44"/>
+    </row>
+    <row r="20" spans="1:14" s="48" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="47"/>
+      <c r="B20" s="127" t="s">
         <v>66</v>
       </c>
-      <c r="C20" s="69"/>
-      <c r="D20" s="70"/>
-      <c r="F20" s="72" t="s">
+      <c r="C20" s="127"/>
+      <c r="D20" s="129"/>
+      <c r="F20" s="49" t="s">
         <v>39</v>
       </c>
-      <c r="G20" s="72"/>
-      <c r="H20" s="72"/>
-      <c r="I20" s="73"/>
-      <c r="J20" s="67"/>
-      <c r="L20" s="74"/>
-      <c r="M20" s="65"/>
-    </row>
-    <row r="21" spans="1:14" s="71" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="75"/>
-      <c r="B21" s="76"/>
-      <c r="C21" s="76"/>
-      <c r="D21" s="77"/>
-      <c r="F21" s="57" t="s">
+      <c r="G20" s="49"/>
+      <c r="H20" s="49"/>
+      <c r="I20" s="50"/>
+      <c r="J20" s="46"/>
+      <c r="L20" s="51"/>
+      <c r="M20" s="44"/>
+    </row>
+    <row r="21" spans="1:14" s="48" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="52"/>
+      <c r="B21" s="128"/>
+      <c r="C21" s="128"/>
+      <c r="D21" s="130"/>
+      <c r="F21" s="132" t="s">
         <v>79</v>
       </c>
-      <c r="G21" s="58"/>
-      <c r="H21" s="59"/>
-      <c r="I21" s="73"/>
-      <c r="J21" s="67"/>
-      <c r="L21" s="74"/>
-      <c r="M21" s="65"/>
-    </row>
-    <row r="22" spans="1:14" s="71" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="75"/>
-      <c r="B22" s="73"/>
-      <c r="C22" s="73"/>
-      <c r="D22" s="53"/>
-      <c r="I22" s="73"/>
-      <c r="J22" s="67"/>
-      <c r="L22" s="74"/>
-      <c r="M22" s="65"/>
+      <c r="G21" s="133"/>
+      <c r="H21" s="134"/>
+      <c r="I21" s="50"/>
+      <c r="J21" s="46"/>
+      <c r="L21" s="51"/>
+      <c r="M21" s="44"/>
+    </row>
+    <row r="22" spans="1:14" s="48" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="52"/>
+      <c r="B22" s="50"/>
+      <c r="C22" s="50"/>
+      <c r="D22" s="42"/>
+      <c r="I22" s="50"/>
+      <c r="J22" s="46"/>
+      <c r="L22" s="51"/>
+      <c r="M22" s="44"/>
     </row>
     <row r="23" spans="1:14" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="78"/>
-      <c r="B23" s="79"/>
-      <c r="C23" s="79"/>
-      <c r="D23" s="79"/>
-      <c r="E23" s="79"/>
-      <c r="F23" s="79"/>
-      <c r="G23" s="79"/>
-      <c r="H23" s="79"/>
-      <c r="I23" s="79"/>
-      <c r="J23" s="80"/>
-      <c r="L23" s="134"/>
+      <c r="A23" s="53"/>
+      <c r="B23" s="54"/>
+      <c r="C23" s="54"/>
+      <c r="D23" s="54"/>
+      <c r="E23" s="54"/>
+      <c r="F23" s="54"/>
+      <c r="G23" s="54"/>
+      <c r="H23" s="54"/>
+      <c r="I23" s="54"/>
+      <c r="J23" s="55"/>
+      <c r="L23" s="95"/>
     </row>
     <row r="24" spans="1:14" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="81"/>
-      <c r="B24" s="81"/>
-      <c r="J24" s="81"/>
-      <c r="K24" s="34"/>
-      <c r="L24" s="135"/>
+      <c r="A24" s="56"/>
+      <c r="B24" s="56"/>
+      <c r="J24" s="56"/>
+      <c r="K24" s="30"/>
+      <c r="L24" s="96"/>
     </row>
     <row r="25" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="82" t="s">
+      <c r="A25" s="57" t="s">
         <v>40</v>
       </c>
-      <c r="B25" s="83" t="s">
+      <c r="B25" s="58" t="s">
         <v>57</v>
       </c>
-      <c r="C25" s="84"/>
-      <c r="D25" s="84"/>
-      <c r="E25" s="84"/>
-      <c r="F25" s="84"/>
-      <c r="G25" s="85"/>
-      <c r="H25" s="86" t="s">
+      <c r="C25" s="59"/>
+      <c r="D25" s="59"/>
+      <c r="E25" s="59"/>
+      <c r="F25" s="59"/>
+      <c r="G25" s="60"/>
+      <c r="H25" s="61" t="s">
         <v>54</v>
       </c>
-      <c r="I25" s="86" t="s">
+      <c r="I25" s="61" t="s">
         <v>55</v>
       </c>
-      <c r="J25" s="87" t="s">
+      <c r="J25" s="62" t="s">
         <v>56</v>
       </c>
-      <c r="K25" s="88"/>
-      <c r="L25" s="89"/>
+      <c r="K25" s="63"/>
+      <c r="L25" s="64"/>
     </row>
     <row r="26" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="90" t="s">
+      <c r="A26" s="65" t="s">
         <v>44</v>
       </c>
-      <c r="B26" s="91" t="s">
+      <c r="B26" s="66" t="s">
         <v>26</v>
       </c>
-      <c r="C26" s="92"/>
-      <c r="D26" s="92"/>
-      <c r="E26" s="93"/>
-      <c r="F26" s="93"/>
-      <c r="G26" s="94" t="s">
+      <c r="C26" s="67"/>
+      <c r="D26" s="67"/>
+      <c r="E26" s="68"/>
+      <c r="F26" s="68"/>
+      <c r="G26" s="69" t="s">
         <v>31</v>
       </c>
       <c r="H26" s="13">
@@ -2526,519 +2520,518 @@
         <f>+H26+0.0045</f>
         <v>4.4999999999999997E-3</v>
       </c>
-      <c r="K26" s="95"/>
-      <c r="L26" s="137"/>
-      <c r="N26" s="136"/>
+      <c r="K26" s="70"/>
+      <c r="N26" s="97"/>
     </row>
     <row r="27" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="90" t="s">
+      <c r="A27" s="65" t="s">
         <v>45</v>
       </c>
-      <c r="B27" s="91" t="s">
+      <c r="B27" s="66" t="s">
         <v>27</v>
       </c>
-      <c r="C27" s="92"/>
-      <c r="D27" s="92"/>
-      <c r="E27" s="93"/>
-      <c r="F27" s="93"/>
-      <c r="G27" s="94" t="s">
+      <c r="C27" s="67"/>
+      <c r="D27" s="67"/>
+      <c r="E27" s="68"/>
+      <c r="F27" s="68"/>
+      <c r="G27" s="69" t="s">
         <v>31</v>
       </c>
-      <c r="H27" s="96">
+      <c r="H27" s="71">
         <f>H26+L27</f>
         <v>0</v>
       </c>
-      <c r="I27" s="96">
+      <c r="I27" s="71">
         <f>I26+L27</f>
         <v>2.5000000000000001E-3</v>
       </c>
-      <c r="J27" s="96">
+      <c r="J27" s="71">
         <f>J26+L27</f>
         <v>4.4999999999999997E-3</v>
       </c>
-      <c r="K27" s="97"/>
-      <c r="L27" s="136"/>
+      <c r="K27" s="72"/>
+      <c r="L27" s="97"/>
     </row>
     <row r="28" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="90" t="s">
+      <c r="A28" s="65" t="s">
         <v>46</v>
       </c>
-      <c r="B28" s="91" t="s">
+      <c r="B28" s="66" t="s">
         <v>42</v>
       </c>
-      <c r="C28" s="92"/>
-      <c r="D28" s="92"/>
-      <c r="E28" s="93"/>
-      <c r="F28" s="93"/>
-      <c r="G28" s="94" t="s">
+      <c r="C28" s="67"/>
+      <c r="D28" s="67"/>
+      <c r="E28" s="68"/>
+      <c r="F28" s="68"/>
+      <c r="G28" s="69" t="s">
         <v>31</v>
       </c>
-      <c r="H28" s="98">
+      <c r="H28" s="73">
         <v>10</v>
       </c>
-      <c r="I28" s="98">
+      <c r="I28" s="73">
         <v>10</v>
       </c>
-      <c r="J28" s="98">
+      <c r="J28" s="73">
         <v>10</v>
       </c>
-      <c r="K28" s="99"/>
-      <c r="L28" s="136"/>
+      <c r="K28" s="74"/>
+      <c r="L28" s="97"/>
     </row>
     <row r="29" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="90" t="s">
+      <c r="A29" s="65" t="s">
         <v>47</v>
       </c>
-      <c r="B29" s="91" t="s">
+      <c r="B29" s="66" t="s">
         <v>43</v>
       </c>
-      <c r="C29" s="92"/>
-      <c r="D29" s="92"/>
-      <c r="E29" s="93"/>
-      <c r="F29" s="93"/>
-      <c r="G29" s="94" t="s">
+      <c r="C29" s="67"/>
+      <c r="D29" s="67"/>
+      <c r="E29" s="68"/>
+      <c r="F29" s="68"/>
+      <c r="G29" s="69" t="s">
         <v>41</v>
       </c>
-      <c r="H29" s="98">
+      <c r="H29" s="73">
         <v>45</v>
       </c>
-      <c r="I29" s="98">
+      <c r="I29" s="73">
         <v>45</v>
       </c>
-      <c r="J29" s="98">
+      <c r="J29" s="73">
         <v>45</v>
       </c>
-      <c r="K29" s="99"/>
-      <c r="L29" s="138"/>
+      <c r="K29" s="74"/>
+      <c r="L29" s="95"/>
     </row>
     <row r="30" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="90" t="s">
+      <c r="A30" s="65" t="s">
         <v>12</v>
       </c>
-      <c r="B30" s="91" t="s">
+      <c r="B30" s="66" t="s">
         <v>28</v>
       </c>
-      <c r="C30" s="92"/>
-      <c r="D30" s="92"/>
-      <c r="E30" s="93"/>
-      <c r="F30" s="93"/>
-      <c r="G30" s="94" t="s">
+      <c r="C30" s="67"/>
+      <c r="D30" s="67"/>
+      <c r="E30" s="68"/>
+      <c r="F30" s="68"/>
+      <c r="G30" s="69" t="s">
         <v>31</v>
       </c>
-      <c r="H30" s="96">
+      <c r="H30" s="71">
         <f>H27+N26</f>
         <v>0</v>
       </c>
-      <c r="I30" s="96">
+      <c r="I30" s="71">
         <f>I27+N26</f>
         <v>2.5000000000000001E-3</v>
       </c>
-      <c r="J30" s="96">
+      <c r="J30" s="71">
         <f>J27+N26</f>
         <v>4.4999999999999997E-3</v>
       </c>
-      <c r="K30" s="99"/>
-      <c r="L30" s="34"/>
+      <c r="K30" s="74"/>
+      <c r="L30" s="30"/>
     </row>
     <row r="31" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="90" t="s">
+      <c r="A31" s="65" t="s">
         <v>13</v>
       </c>
-      <c r="B31" s="91" t="s">
+      <c r="B31" s="66" t="s">
         <v>29</v>
       </c>
-      <c r="C31" s="92"/>
-      <c r="D31" s="92"/>
-      <c r="E31" s="93"/>
-      <c r="F31" s="93"/>
-      <c r="G31" s="94" t="s">
+      <c r="C31" s="67"/>
+      <c r="D31" s="67"/>
+      <c r="E31" s="68"/>
+      <c r="F31" s="68"/>
+      <c r="G31" s="69" t="s">
         <v>31</v>
       </c>
-      <c r="H31" s="96">
+      <c r="H31" s="71">
         <f>IF(H30=0,0,H30+L28)</f>
         <v>0</v>
       </c>
-      <c r="I31" s="96">
+      <c r="I31" s="71">
         <f>IF(I30=0,0,I30+L28)</f>
         <v>2.5000000000000001E-3</v>
       </c>
-      <c r="J31" s="96">
+      <c r="J31" s="71">
         <f>IF(J30=0,0,J30+L28)</f>
         <v>4.4999999999999997E-3</v>
       </c>
-      <c r="K31" s="99"/>
-      <c r="L31" s="34"/>
+      <c r="K31" s="74"/>
+      <c r="L31" s="30"/>
     </row>
     <row r="32" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="90" t="s">
+      <c r="A32" s="65" t="s">
         <v>48</v>
       </c>
-      <c r="B32" s="91" t="s">
+      <c r="B32" s="66" t="s">
         <v>36</v>
       </c>
-      <c r="C32" s="92"/>
-      <c r="D32" s="92"/>
-      <c r="E32" s="93"/>
-      <c r="F32" s="93"/>
-      <c r="G32" s="94" t="s">
+      <c r="C32" s="67"/>
+      <c r="D32" s="67"/>
+      <c r="E32" s="68"/>
+      <c r="F32" s="68"/>
+      <c r="G32" s="69" t="s">
         <v>18</v>
       </c>
-      <c r="H32" s="98">
+      <c r="H32" s="73">
         <v>20</v>
       </c>
-      <c r="I32" s="98">
+      <c r="I32" s="73">
         <v>20</v>
       </c>
-      <c r="J32" s="98">
+      <c r="J32" s="73">
         <v>20</v>
       </c>
-      <c r="K32" s="100"/>
-      <c r="L32" s="34"/>
+      <c r="K32" s="75"/>
+      <c r="L32" s="30"/>
     </row>
     <row r="33" spans="1:12" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="90" t="s">
+      <c r="A33" s="65" t="s">
         <v>49</v>
       </c>
-      <c r="B33" s="101" t="s">
+      <c r="B33" s="76" t="s">
         <v>33</v>
       </c>
-      <c r="C33" s="92"/>
-      <c r="D33" s="92"/>
-      <c r="E33" s="102"/>
-      <c r="F33" s="102"/>
-      <c r="G33" s="94" t="s">
+      <c r="C33" s="67"/>
+      <c r="D33" s="67"/>
+      <c r="E33" s="77"/>
+      <c r="F33" s="77"/>
+      <c r="G33" s="69" t="s">
         <v>32</v>
       </c>
-      <c r="H33" s="103">
+      <c r="H33" s="136">
         <v>11.5</v>
       </c>
-      <c r="I33" s="103">
+      <c r="I33" s="136">
         <v>11.7</v>
       </c>
-      <c r="J33" s="103">
+      <c r="J33" s="136">
         <v>11.8</v>
       </c>
-      <c r="K33" s="104"/>
-      <c r="L33" s="34"/>
+      <c r="K33" s="78"/>
+      <c r="L33" s="30"/>
     </row>
     <row r="34" spans="1:12" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="90" t="s">
+      <c r="A34" s="65" t="s">
         <v>50</v>
       </c>
-      <c r="B34" s="101" t="s">
+      <c r="B34" s="76" t="s">
         <v>34</v>
       </c>
-      <c r="C34" s="92"/>
-      <c r="D34" s="92"/>
-      <c r="E34" s="105"/>
-      <c r="F34" s="105"/>
-      <c r="G34" s="94" t="s">
+      <c r="C34" s="67"/>
+      <c r="D34" s="67"/>
+      <c r="E34" s="79"/>
+      <c r="F34" s="79"/>
+      <c r="G34" s="69" t="s">
         <v>32</v>
       </c>
-      <c r="H34" s="103">
+      <c r="H34" s="136">
         <v>2.9</v>
       </c>
-      <c r="I34" s="103">
+      <c r="I34" s="136">
         <v>2.7</v>
       </c>
-      <c r="J34" s="103">
+      <c r="J34" s="136">
         <v>2.8</v>
       </c>
-      <c r="K34" s="106"/>
-      <c r="L34" s="34"/>
+      <c r="K34" s="80"/>
+      <c r="L34" s="30"/>
     </row>
     <row r="35" spans="1:12" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="90" t="s">
+      <c r="A35" s="65" t="s">
         <v>51</v>
       </c>
-      <c r="B35" s="101" t="s">
+      <c r="B35" s="76" t="s">
         <v>53</v>
       </c>
-      <c r="C35" s="92"/>
-      <c r="D35" s="92"/>
-      <c r="E35" s="105"/>
-      <c r="F35" s="105"/>
-      <c r="G35" s="94" t="s">
+      <c r="C35" s="67"/>
+      <c r="D35" s="67"/>
+      <c r="E35" s="79"/>
+      <c r="F35" s="79"/>
+      <c r="G35" s="69" t="s">
         <v>17</v>
       </c>
-      <c r="H35" s="130">
+      <c r="H35" s="94">
         <f>ROUNDUP((H34/H33*100),0)</f>
         <v>26</v>
       </c>
-      <c r="I35" s="130">
+      <c r="I35" s="94">
         <f t="shared" ref="I35:J35" si="0">ROUNDUP((I34/I33*100),0)</f>
         <v>24</v>
       </c>
-      <c r="J35" s="130">
+      <c r="J35" s="94">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="K35" s="34"/>
-      <c r="L35" s="34"/>
+      <c r="K35" s="30"/>
+      <c r="L35" s="30"/>
     </row>
     <row r="36" spans="1:12" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="90" t="s">
+      <c r="A36" s="65" t="s">
         <v>52</v>
       </c>
-      <c r="B36" s="107" t="s">
+      <c r="B36" s="81" t="s">
         <v>35</v>
       </c>
-      <c r="C36" s="92"/>
-      <c r="D36" s="92"/>
-      <c r="E36" s="105"/>
-      <c r="F36" s="105"/>
-      <c r="G36" s="94" t="s">
+      <c r="C36" s="67"/>
+      <c r="D36" s="67"/>
+      <c r="E36" s="79"/>
+      <c r="F36" s="79"/>
+      <c r="G36" s="69" t="s">
         <v>17</v>
       </c>
-      <c r="H36" s="131">
+      <c r="H36" s="119">
         <f>ROUNDUP((AVERAGE(H35:J35)),0)</f>
         <v>25</v>
       </c>
-      <c r="I36" s="132"/>
-      <c r="J36" s="133"/>
-      <c r="K36" s="34"/>
-      <c r="L36" s="34"/>
+      <c r="I36" s="120"/>
+      <c r="J36" s="121"/>
+      <c r="K36" s="30"/>
+      <c r="L36" s="30"/>
     </row>
     <row r="37" spans="1:12" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="108"/>
-      <c r="B37" s="108"/>
-      <c r="C37" s="109"/>
-      <c r="D37" s="110"/>
-      <c r="E37" s="110"/>
-      <c r="F37" s="110"/>
-      <c r="G37" s="110"/>
-      <c r="H37" s="110"/>
-      <c r="I37" s="110"/>
-      <c r="J37" s="111"/>
-      <c r="K37" s="34"/>
-      <c r="L37" s="34"/>
+      <c r="A37" s="82"/>
+      <c r="B37" s="82"/>
+      <c r="C37" s="83"/>
+      <c r="D37" s="84"/>
+      <c r="E37" s="84"/>
+      <c r="F37" s="84"/>
+      <c r="G37" s="84"/>
+      <c r="H37" s="84"/>
+      <c r="I37" s="84"/>
+      <c r="J37" s="85"/>
+      <c r="K37" s="30"/>
+      <c r="L37" s="30"/>
     </row>
     <row r="38" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="112" t="s">
+      <c r="A38" s="114" t="s">
         <v>22</v>
       </c>
-      <c r="B38" s="113"/>
-      <c r="C38" s="114"/>
-      <c r="D38" s="112" t="s">
+      <c r="B38" s="116"/>
+      <c r="C38" s="115"/>
+      <c r="D38" s="114" t="s">
         <v>23</v>
       </c>
-      <c r="E38" s="114"/>
-      <c r="F38" s="115" t="s">
+      <c r="E38" s="115"/>
+      <c r="F38" s="86" t="s">
         <v>20</v>
       </c>
-      <c r="G38" s="116"/>
-      <c r="H38" s="116"/>
-      <c r="I38" s="116"/>
-      <c r="J38" s="117"/>
-      <c r="K38" s="34"/>
-      <c r="L38" s="34"/>
+      <c r="G38" s="87"/>
+      <c r="H38" s="87"/>
+      <c r="I38" s="87"/>
+      <c r="J38" s="88"/>
+      <c r="K38" s="30"/>
+      <c r="L38" s="30"/>
     </row>
     <row r="39" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="118" t="s">
+      <c r="A39" s="108" t="s">
         <v>24</v>
       </c>
-      <c r="B39" s="119"/>
-      <c r="C39" s="120"/>
-      <c r="D39" s="118" t="s">
+      <c r="B39" s="109"/>
+      <c r="C39" s="110"/>
+      <c r="D39" s="108" t="s">
         <v>69</v>
       </c>
-      <c r="E39" s="120"/>
-      <c r="F39" s="78"/>
-      <c r="G39" s="79"/>
-      <c r="H39" s="79"/>
-      <c r="I39" s="79"/>
-      <c r="J39" s="80"/>
-      <c r="K39" s="34"/>
-      <c r="L39" s="34"/>
+      <c r="E39" s="110"/>
+      <c r="F39" s="53"/>
+      <c r="G39" s="54"/>
+      <c r="H39" s="54"/>
+      <c r="I39" s="54"/>
+      <c r="J39" s="55"/>
+      <c r="K39" s="30"/>
+      <c r="L39" s="30"/>
     </row>
     <row r="40" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="118" t="s">
+      <c r="A40" s="108" t="s">
         <v>25</v>
       </c>
-      <c r="B40" s="119"/>
-      <c r="C40" s="120"/>
-      <c r="D40" s="118" t="s">
+      <c r="B40" s="109"/>
+      <c r="C40" s="110"/>
+      <c r="D40" s="108" t="s">
         <v>67</v>
       </c>
-      <c r="E40" s="120"/>
-      <c r="F40" s="121"/>
-      <c r="G40" s="116"/>
-      <c r="H40" s="116"/>
-      <c r="I40" s="116"/>
-      <c r="J40" s="116"/>
-      <c r="K40" s="34"/>
-      <c r="L40" s="34"/>
+      <c r="E40" s="110"/>
+      <c r="F40" s="89"/>
+      <c r="G40" s="87"/>
+      <c r="H40" s="87"/>
+      <c r="I40" s="87"/>
+      <c r="J40" s="87"/>
+      <c r="K40" s="30"/>
+      <c r="L40" s="30"/>
     </row>
     <row r="41" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="118" t="s">
+      <c r="A41" s="108" t="s">
         <v>63</v>
       </c>
-      <c r="B41" s="119"/>
-      <c r="C41" s="120"/>
-      <c r="D41" s="118" t="s">
+      <c r="B41" s="109"/>
+      <c r="C41" s="110"/>
+      <c r="D41" s="108" t="s">
         <v>70</v>
       </c>
-      <c r="E41" s="120"/>
-      <c r="F41" s="51"/>
-      <c r="K41" s="34"/>
-      <c r="L41" s="34"/>
+      <c r="E41" s="110"/>
+      <c r="F41" s="41"/>
+      <c r="K41" s="30"/>
+      <c r="L41" s="30"/>
     </row>
     <row r="42" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="122" t="s">
+      <c r="A42" s="111" t="s">
         <v>62</v>
       </c>
-      <c r="B42" s="123"/>
-      <c r="C42" s="124"/>
-      <c r="D42" s="118" t="s">
+      <c r="B42" s="112"/>
+      <c r="C42" s="113"/>
+      <c r="D42" s="108" t="s">
         <v>68</v>
       </c>
-      <c r="E42" s="120"/>
-      <c r="F42" s="51"/>
-      <c r="K42" s="34"/>
-      <c r="L42" s="34"/>
+      <c r="E42" s="110"/>
+      <c r="F42" s="41"/>
+      <c r="K42" s="30"/>
+      <c r="L42" s="30"/>
     </row>
     <row r="43" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="122" t="s">
+      <c r="A43" s="111" t="s">
         <v>64</v>
       </c>
-      <c r="B43" s="123"/>
-      <c r="C43" s="124"/>
-      <c r="D43" s="118" t="s">
+      <c r="B43" s="112"/>
+      <c r="C43" s="113"/>
+      <c r="D43" s="108" t="s">
         <v>71</v>
       </c>
-      <c r="E43" s="120"/>
-      <c r="F43" s="51"/>
-      <c r="K43" s="34"/>
-      <c r="L43" s="34"/>
+      <c r="E43" s="110"/>
+      <c r="F43" s="41"/>
+      <c r="K43" s="30"/>
+      <c r="L43" s="30"/>
     </row>
     <row r="44" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="118" t="s">
+      <c r="A44" s="108" t="s">
         <v>59</v>
       </c>
-      <c r="B44" s="119"/>
-      <c r="C44" s="120"/>
-      <c r="D44" s="118" t="s">
+      <c r="B44" s="109"/>
+      <c r="C44" s="110"/>
+      <c r="D44" s="108" t="s">
         <v>72</v>
       </c>
-      <c r="E44" s="120"/>
-      <c r="F44" s="51"/>
-      <c r="K44" s="34"/>
-      <c r="L44" s="34"/>
+      <c r="E44" s="110"/>
+      <c r="F44" s="41"/>
+      <c r="K44" s="30"/>
+      <c r="L44" s="30"/>
     </row>
     <row r="45" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="118" t="s">
+      <c r="A45" s="108" t="s">
         <v>77</v>
       </c>
-      <c r="B45" s="119"/>
-      <c r="C45" s="120"/>
-      <c r="D45" s="118" t="s">
+      <c r="B45" s="109"/>
+      <c r="C45" s="110"/>
+      <c r="D45" s="108" t="s">
         <v>78</v>
       </c>
-      <c r="E45" s="120"/>
-      <c r="F45" s="51"/>
-      <c r="K45" s="34"/>
-      <c r="L45" s="34"/>
+      <c r="E45" s="110"/>
+      <c r="F45" s="41"/>
+      <c r="K45" s="30"/>
+      <c r="L45" s="30"/>
     </row>
     <row r="46" spans="1:12" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="125"/>
-      <c r="B46" s="125"/>
-      <c r="C46" s="111"/>
-      <c r="D46" s="111"/>
-      <c r="E46" s="111"/>
-      <c r="F46" s="111"/>
-      <c r="G46" s="111"/>
-      <c r="H46" s="111"/>
-      <c r="I46" s="111"/>
-      <c r="J46" s="111"/>
-      <c r="K46" s="34"/>
-      <c r="L46" s="34"/>
+      <c r="A46" s="90"/>
+      <c r="B46" s="90"/>
+      <c r="C46" s="85"/>
+      <c r="D46" s="85"/>
+      <c r="E46" s="85"/>
+      <c r="F46" s="85"/>
+      <c r="G46" s="85"/>
+      <c r="H46" s="85"/>
+      <c r="I46" s="85"/>
+      <c r="J46" s="85"/>
+      <c r="K46" s="30"/>
+      <c r="L46" s="30"/>
     </row>
     <row r="47" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="126"/>
-      <c r="B47" s="126"/>
-      <c r="C47" s="111"/>
-      <c r="J47" s="111"/>
-      <c r="K47" s="34"/>
-      <c r="L47" s="34"/>
+      <c r="A47" s="91"/>
+      <c r="B47" s="91"/>
+      <c r="C47" s="85"/>
+      <c r="J47" s="85"/>
+      <c r="K47" s="30"/>
+      <c r="L47" s="30"/>
     </row>
     <row r="48" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="126"/>
-      <c r="B48" s="126"/>
-      <c r="C48" s="111"/>
-      <c r="J48" s="111"/>
-      <c r="K48" s="34"/>
-      <c r="L48" s="34"/>
+      <c r="A48" s="91"/>
+      <c r="B48" s="91"/>
+      <c r="C48" s="85"/>
+      <c r="J48" s="85"/>
+      <c r="K48" s="30"/>
+      <c r="L48" s="30"/>
     </row>
     <row r="49" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="126"/>
-      <c r="B49" s="126"/>
-      <c r="C49" s="111"/>
-      <c r="J49" s="111"/>
-      <c r="K49" s="34"/>
-      <c r="L49" s="34"/>
+      <c r="A49" s="91"/>
+      <c r="B49" s="91"/>
+      <c r="C49" s="85"/>
+      <c r="J49" s="85"/>
+      <c r="K49" s="30"/>
+      <c r="L49" s="30"/>
     </row>
     <row r="50" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="127"/>
-      <c r="B50" s="127"/>
-      <c r="C50" s="111"/>
-      <c r="D50" s="111"/>
-      <c r="E50" s="111"/>
-      <c r="F50" s="111"/>
-      <c r="G50" s="111"/>
-      <c r="H50" s="111"/>
-      <c r="I50" s="111"/>
-      <c r="J50" s="111"/>
-      <c r="K50" s="34"/>
-      <c r="L50" s="34"/>
+      <c r="A50" s="92"/>
+      <c r="B50" s="92"/>
+      <c r="C50" s="85"/>
+      <c r="D50" s="85"/>
+      <c r="E50" s="85"/>
+      <c r="F50" s="85"/>
+      <c r="G50" s="85"/>
+      <c r="H50" s="85"/>
+      <c r="I50" s="85"/>
+      <c r="J50" s="85"/>
+      <c r="K50" s="30"/>
+      <c r="L50" s="30"/>
     </row>
     <row r="51" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="128" t="s">
+      <c r="A51" s="93" t="s">
         <v>16</v>
       </c>
-      <c r="B51" s="128"/>
-      <c r="C51" s="111"/>
-      <c r="D51" s="111"/>
-      <c r="E51" s="111"/>
-      <c r="F51" s="111"/>
-      <c r="G51" s="111"/>
-      <c r="H51" s="111"/>
-      <c r="I51" s="111"/>
-      <c r="J51" s="111"/>
-      <c r="K51" s="34"/>
-      <c r="L51" s="34"/>
+      <c r="B51" s="93"/>
+      <c r="C51" s="85"/>
+      <c r="D51" s="85"/>
+      <c r="E51" s="85"/>
+      <c r="F51" s="85"/>
+      <c r="G51" s="85"/>
+      <c r="H51" s="85"/>
+      <c r="I51" s="85"/>
+      <c r="J51" s="85"/>
+      <c r="K51" s="30"/>
+      <c r="L51" s="30"/>
     </row>
     <row r="52" spans="1:12" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="128" t="s">
+      <c r="A52" s="93" t="s">
         <v>65</v>
       </c>
-      <c r="B52" s="128"/>
-      <c r="C52" s="111"/>
-      <c r="D52" s="111"/>
-      <c r="E52" s="111"/>
-      <c r="F52" s="97" t="s">
+      <c r="B52" s="93"/>
+      <c r="C52" s="85"/>
+      <c r="D52" s="85"/>
+      <c r="E52" s="85"/>
+      <c r="F52" s="72" t="s">
         <v>30</v>
       </c>
-      <c r="G52" s="111"/>
-      <c r="H52" s="111"/>
-      <c r="I52" s="111"/>
-      <c r="J52" s="111"/>
-      <c r="K52" s="34"/>
-      <c r="L52" s="34"/>
+      <c r="G52" s="85"/>
+      <c r="H52" s="85"/>
+      <c r="I52" s="85"/>
+      <c r="J52" s="85"/>
+      <c r="K52" s="30"/>
+      <c r="L52" s="30"/>
     </row>
     <row r="53" spans="1:12" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="54" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="129" t="s">
+      <c r="A54" s="98" t="s">
         <v>19</v>
       </c>
-      <c r="B54" s="129"/>
-      <c r="C54" s="129"/>
-      <c r="D54" s="129"/>
-      <c r="E54" s="129"/>
-      <c r="F54" s="129"/>
-      <c r="G54" s="129"/>
-      <c r="H54" s="129"/>
-      <c r="I54" s="129"/>
-      <c r="J54" s="129"/>
+      <c r="B54" s="98"/>
+      <c r="C54" s="98"/>
+      <c r="D54" s="98"/>
+      <c r="E54" s="98"/>
+      <c r="F54" s="98"/>
+      <c r="G54" s="98"/>
+      <c r="H54" s="98"/>
+      <c r="I54" s="98"/>
+      <c r="J54" s="98"/>
     </row>
     <row r="55" spans="1:12" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="56" spans="1:12" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -3050,6 +3043,29 @@
     <protectedRange sqref="H31:J31" name="Rango8_1"/>
   </protectedRanges>
   <mergeCells count="39">
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="A44:C44"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="A7:J7"/>
+    <mergeCell ref="A8:J8"/>
+    <mergeCell ref="H36:J36"/>
+    <mergeCell ref="A13:J13"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="B20:C21"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="F21:H21"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="F17:G17"/>
     <mergeCell ref="A54:J54"/>
     <mergeCell ref="A14:J14"/>
     <mergeCell ref="I16:I18"/>
@@ -3066,29 +3082,6 @@
     <mergeCell ref="A38:C38"/>
     <mergeCell ref="A41:C41"/>
     <mergeCell ref="A42:C42"/>
-    <mergeCell ref="A7:J7"/>
-    <mergeCell ref="A8:J8"/>
-    <mergeCell ref="H36:J36"/>
-    <mergeCell ref="A13:J13"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="F16:G16"/>
-    <mergeCell ref="B20:C21"/>
-    <mergeCell ref="D20:D21"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="F21:H21"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="D41:E41"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="A44:C44"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D11:E11"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
@@ -3116,10 +3109,10 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="135" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="14"/>
+      <c r="B2" s="135"/>
       <c r="C2" s="5" t="s">
         <v>10</v>
       </c>

</xml_diff>